<commit_message>
test  the new method no error
</commit_message>
<xml_diff>
--- a/reports/09_06_2026.xlsx
+++ b/reports/09_06_2026.xlsx
@@ -147,6 +147,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -166,6 +169,171 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2181225" cy="1704975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1028700" cy="485775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2200275" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1038225" cy="447675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2276475" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1009650" cy="581025"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -468,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35.88" customWidth="1" min="6" max="6"/>
@@ -537,6 +705,81 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="134" customHeight="1">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0ALIJI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>09 June 2026  10:52:50  AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="135" customHeight="1">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>09 June 2026  10:52:56  AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="135" customHeight="1">
+      <c r="A5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NDUOU</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>09 June 2026  10:53:01  AM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>